<commit_message>
feat(balance): L01 波次奖励最终 原值+10（W5/10/15/20 原值+35），合计 955→1305
三轮下发累加后定稿：+5/+15 → (替换)+7/+20 → (叠加)+3/+5，即每波 +10、W5/10/15/20 +35。25 行 rewardGold 全改，W1 26→36、W5 49→84、W25 61→71。只动 Level01 的 RoundData，其余 29 关与血量未牵连。Luban 已重导出 tbrounddata.json（25 行差异，增量仅 +10/+35）。
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/Levels/L01/RoundData.xlsx
+++ b/Luban/Config/Datas/Levels/L01/RoundData.xlsx
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="F4" s="0" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="F5" s="0" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="F6" s="0" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="1" s="2">
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>49</v>
+        <v>84</v>
       </c>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
@@ -1446,7 +1446,7 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="F12" s="0" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="L12" s="13" t="n"/>
       <c r="M12" s="13" t="n"/>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="F13" s="0" t="n">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="L13" s="13" t="n"/>
       <c r="M13" s="13" t="n"/>
@@ -1520,7 +1520,7 @@
         </is>
       </c>
       <c r="F14" s="0" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="L14" s="13" t="n"/>
       <c r="M14" s="13" t="n"/>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="F15" s="0" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="L15" s="13" t="n"/>
       <c r="M15" s="13" t="n"/>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="F16" s="0" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" s="1">
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="F17" s="0" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" s="1">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="F18" s="0" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" s="1">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="F19" s="0" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" s="1">
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="F20" s="0" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" s="1">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="F21" s="0" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="F22" s="0" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23">
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="F23" s="0" t="n">
-        <v>55</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24">
@@ -1734,7 +1734,7 @@
         </is>
       </c>
       <c r="F24" s="0" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25">
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="F25" s="0" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26">
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="F26" s="0" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="F27" s="0" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="F28" s="0" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>